<commit_message>
changes which I don't remember
</commit_message>
<xml_diff>
--- a/example_tables/Амортизация_аренда.xlsx
+++ b/example_tables/Амортизация_аренда.xlsx
@@ -923,7 +923,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>ООО КОНТЕНТ</t>
+          <t>ООО Контент</t>
         </is>
       </c>
       <c r="B7" s="5" t="n"/>
@@ -1797,7 +1797,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>ООО ПЕРСПЕКТИВА</t>
+          <t>ООО Перспектива</t>
         </is>
       </c>
       <c r="B24" s="5" t="n"/>

</xml_diff>